<commit_message>
Add custom Metadata API & strict run alignment
Support per-model Metadata API base URLs (e.g., ensemble-api.open-meteo.com for GEM/GEPS) via new `meta_base_url` config field. Enable GEM metadata fetching by adding `cmc_gem_geps` slug.

Introduce CROSS_CHECK_RUN_ALIGN_TOL_H (3h) to enforce strict run_date alignment between xlsx and parquet sources. Skip models with misaligned cycles instead of warning, preventing misleading cross-check comparisons.

Update app version to 2.0.2.
</commit_message>
<xml_diff>
--- a/Forecasts/Forecast-01072026-0Z.xlsx
+++ b/Forecasts/Forecast-01072026-0Z.xlsx
@@ -653,7 +653,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 01/07/2026 11:19</t>
+          <t>Généré le : 01/07/2026 12:04</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 01/07/2026 11:19</t>
+          <t>Généré le : 01/07/2026 12:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MAJ auto données météo
</commit_message>
<xml_diff>
--- a/Forecasts/Forecast-01072026-0Z.xlsx
+++ b/Forecasts/Forecast-01072026-0Z.xlsx
@@ -653,7 +653,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 01/07/2026 09:16</t>
+          <t>Généré le : 01/07/2026 11:14</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 01/07/2026 09:16</t>
+          <t>Généré le : 01/07/2026 11:14</t>
         </is>
       </c>
     </row>

</xml_diff>